<commit_message>
repo autocontenido + docs para retomar: Excel crudos versionados, ESTADO/CONTEXTO/CLAUDE.md, scripts IPC y ejecucion local
- data/raw versionado (sector_publico.zip + 4 meses sueltos 2026); duplicados del ZIP
  quedan locales en data/raw/_duplicados (ignorado). consolidate.py reproduce los CSV byte a byte
- IPC: divisiones jun-ago 2026 completadas
- scripts/actualizar_ipc.py (API datos.gob.ar) y scripts/run_notebooks_local.py
- README reescrito; ESTADO.md (estado + rutina mensual), CONTEXTO.md (metodologia),
  CLAUDE.md (reglas de sesion); memoria de proyecto reorganizada
- requirements: matplotlib, nbconvert, ipykernel
</commit_message>
<xml_diff>
--- a/data/reference/IPC.xlsx
+++ b/data/reference/IPC.xlsx
@@ -15,10 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="mmm&quot;-&quot;yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -5613,6 +5612,42 @@
       <c r="B115" t="n">
         <v>11826.4103</v>
       </c>
+      <c r="C115" t="n">
+        <v>12657.46</v>
+      </c>
+      <c r="D115" t="n">
+        <v>8201.66</v>
+      </c>
+      <c r="E115" t="n">
+        <v>8384.719999999999</v>
+      </c>
+      <c r="F115" t="n">
+        <v>13213.15</v>
+      </c>
+      <c r="G115" t="n">
+        <v>9455.040000000001</v>
+      </c>
+      <c r="H115" t="n">
+        <v>13200.75</v>
+      </c>
+      <c r="I115" t="n">
+        <v>12531.8</v>
+      </c>
+      <c r="J115" t="n">
+        <v>10933.56</v>
+      </c>
+      <c r="K115" t="n">
+        <v>10556.46</v>
+      </c>
+      <c r="L115" t="n">
+        <v>11025.4</v>
+      </c>
+      <c r="M115" t="n">
+        <v>14524.08</v>
+      </c>
+      <c r="N115" t="n">
+        <v>11373.14</v>
+      </c>
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="14" t="n">
@@ -5621,6 +5656,42 @@
       <c r="B116" t="n">
         <v>12076.3937</v>
       </c>
+      <c r="C116" t="n">
+        <v>12907.51</v>
+      </c>
+      <c r="D116" t="n">
+        <v>8325.6</v>
+      </c>
+      <c r="E116" t="n">
+        <v>8272.280000000001</v>
+      </c>
+      <c r="F116" t="n">
+        <v>13505.36</v>
+      </c>
+      <c r="G116" t="n">
+        <v>9653.719999999999</v>
+      </c>
+      <c r="H116" t="n">
+        <v>13536.83</v>
+      </c>
+      <c r="I116" t="n">
+        <v>12767.66</v>
+      </c>
+      <c r="J116" t="n">
+        <v>11194.26</v>
+      </c>
+      <c r="K116" t="n">
+        <v>11085.75</v>
+      </c>
+      <c r="L116" t="n">
+        <v>11235.67</v>
+      </c>
+      <c r="M116" t="n">
+        <v>14923.82</v>
+      </c>
+      <c r="N116" t="n">
+        <v>11628.31</v>
+      </c>
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="14" t="n">
@@ -5628,6 +5699,42 @@
       </c>
       <c r="B117" t="n">
         <v>12276.766</v>
+      </c>
+      <c r="C117" t="n">
+        <v>13121.25</v>
+      </c>
+      <c r="D117" t="n">
+        <v>8502.120000000001</v>
+      </c>
+      <c r="E117" t="n">
+        <v>8218.76</v>
+      </c>
+      <c r="F117" t="n">
+        <v>13885.49</v>
+      </c>
+      <c r="G117" t="n">
+        <v>9793.690000000001</v>
+      </c>
+      <c r="H117" t="n">
+        <v>13863.05</v>
+      </c>
+      <c r="I117" t="n">
+        <v>12965.12</v>
+      </c>
+      <c r="J117" t="n">
+        <v>11449.47</v>
+      </c>
+      <c r="K117" t="n">
+        <v>11084.1</v>
+      </c>
+      <c r="L117" t="n">
+        <v>11519.72</v>
+      </c>
+      <c r="M117" t="n">
+        <v>15196.18</v>
+      </c>
+      <c r="N117" t="n">
+        <v>11911.9</v>
       </c>
     </row>
     <row r="118" ht="15.75" customHeight="1"/>

</xml_diff>